<commit_message>
Export TRP results to Excel template
</commit_message>
<xml_diff>
--- a/public/report-generator-template.xlsx
+++ b/public/report-generator-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abyos\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://aradtech-my.sharepoint.com/personal/yossef_abutbul_aradtec_com/Documents/Documents/GitHub/ReportGen2/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{241B28CC-6B6E-4F50-ADF8-AA2AB74E77A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{241B28CC-6B6E-4F50-ADF8-AA2AB74E77A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{906503F2-951E-4225-99FA-CADA65535DDC}"/>
   <bookViews>
-    <workbookView xWindow="4980" yWindow="4995" windowWidth="28800" windowHeight="15435" xr2:uid="{ECEE3F40-80EB-4313-9D59-FED83186C7B1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ECEE3F40-80EB-4313-9D59-FED83186C7B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,15 +29,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Unit ID</t>
   </si>
@@ -60,22 +57,7 @@
     <t>Cell Factor</t>
   </si>
   <si>
-    <t>70B3D5A9F017C80F</t>
-  </si>
-  <si>
-    <t>70B3D5A9F013DE16</t>
-  </si>
-  <si>
-    <t>70B3D5A9F0173333</t>
-  </si>
-  <si>
-    <t>70B3D5A9F013DE18</t>
-  </si>
-  <si>
     <t>Unit Type 1</t>
-  </si>
-  <si>
-    <t>Unit Type 2</t>
   </si>
 </sst>
 </file>
@@ -86,7 +68,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -94,14 +76,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -277,17 +259,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
-<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <rel r:id="rId1"/>
-  <rel r:id="rId2"/>
-  <rel r:id="rId3"/>
-  <rel r:id="rId4"/>
-  <rel r:id="rId5"/>
-  <rel r:id="rId6"/>
-</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -608,30 +579,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04346829-E6E2-438D-B519-5766F1E0B38D}">
   <dimension ref="A1:L24"/>
-  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="36.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="36.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.75" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.375" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.125" style="3"/>
-    <col min="7" max="10" width="9.125" style="2"/>
-    <col min="11" max="11" width="11.875" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.125" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="9.125" style="2"/>
+    <col min="5" max="5" width="12.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" style="3"/>
+    <col min="7" max="10" width="9.140625" style="2"/>
+    <col min="11" max="11" width="11.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
       <c r="D1" s="10"/>
       <c r="E1" s="10"/>
     </row>
-    <row r="2" spans="1:12" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
@@ -654,22 +625,17 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="12" t="s">
-        <v>7</v>
-      </c>
+    <row r="3" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="12"/>
       <c r="B3" s="4">
         <v>915.2</v>
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4">
         <f>F3+$L$3</f>
-        <v>18.416999999999998</v>
+        <v>35.976999999999997</v>
       </c>
       <c r="E3" s="4"/>
-      <c r="F3" s="3">
-        <v>-17.559999999999999</v>
-      </c>
       <c r="K3" s="2">
         <v>915.2</v>
       </c>
@@ -677,7 +643,7 @@
         <v>35.976999999999997</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="13"/>
       <c r="B4" s="5">
         <v>922.2</v>
@@ -685,12 +651,9 @@
       <c r="C4" s="5"/>
       <c r="D4" s="5">
         <f>F4+$L$4</f>
-        <v>17.553999999999998</v>
+        <v>35.933999999999997</v>
       </c>
       <c r="E4" s="5"/>
-      <c r="F4" s="3">
-        <v>-18.38</v>
-      </c>
       <c r="K4" s="2">
         <v>922.2</v>
       </c>
@@ -698,7 +661,7 @@
         <v>35.933999999999997</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="14"/>
       <c r="B5" s="6">
         <v>927.8</v>
@@ -706,12 +669,9 @@
       <c r="C5" s="6"/>
       <c r="D5" s="6">
         <f>F5+$L$5</f>
-        <v>16.714000000000002</v>
+        <v>35.804000000000002</v>
       </c>
       <c r="E5" s="6"/>
-      <c r="F5" s="3">
-        <v>-19.09</v>
-      </c>
       <c r="K5" s="2">
         <v>927.8</v>
       </c>
@@ -719,10 +679,8 @@
         <v>35.804000000000002</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="12" t="s">
-        <v>9</v>
-      </c>
+    <row r="6" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12"/>
       <c r="B6" s="4">
         <v>915.2</v>
       </c>
@@ -733,7 +691,7 @@
       </c>
       <c r="E6" s="4"/>
     </row>
-    <row r="7" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="13"/>
       <c r="B7" s="5">
         <v>922.2</v>
@@ -745,7 +703,7 @@
       </c>
       <c r="E7" s="5"/>
     </row>
-    <row r="8" spans="1:12" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14"/>
       <c r="B8" s="6">
         <v>927.8</v>
@@ -757,195 +715,116 @@
       </c>
       <c r="E8" s="6"/>
     </row>
-    <row r="10" spans="1:12" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-    </row>
-    <row r="11" spans="1:12" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12" s="4">
-        <v>915.2</v>
-      </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4">
-        <f>F12+$L$3</f>
-        <v>19.296999999999997</v>
-      </c>
-      <c r="E12" s="4"/>
-      <c r="F12" s="3">
-        <v>-16.68</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="13"/>
-      <c r="B13" s="5">
-        <v>922.2</v>
-      </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5">
-        <f>F13+$L$4</f>
-        <v>19.333999999999996</v>
-      </c>
-      <c r="E13" s="5"/>
-      <c r="F13" s="3">
-        <v>-16.600000000000001</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="14"/>
-      <c r="B14" s="6">
-        <v>927.8</v>
-      </c>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6">
-        <f>F14+$L$5</f>
-        <v>19.124000000000002</v>
-      </c>
-      <c r="E14" s="6"/>
-      <c r="F14" s="3">
-        <v>-16.68</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B15" s="4">
-        <v>915.2</v>
-      </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4">
-        <f>F15+$L$3</f>
-        <v>19.296999999999997</v>
-      </c>
-      <c r="E15" s="4"/>
-      <c r="F15" s="3">
-        <v>-16.68</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="13"/>
-      <c r="B16" s="5">
-        <v>922.2</v>
-      </c>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5">
-        <f>F16+$L$4</f>
-        <v>19.333999999999996</v>
-      </c>
-      <c r="E16" s="5"/>
-      <c r="F16" s="3">
-        <v>-16.600000000000001</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="14"/>
-      <c r="B17" s="6">
-        <v>927.8</v>
-      </c>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6">
-        <f>F17+$L$5</f>
-        <v>19.124000000000002</v>
-      </c>
-      <c r="E17" s="6"/>
-      <c r="F17" s="3">
-        <v>-16.68</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B18" s="4">
-        <v>915.2</v>
-      </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4">
-        <f>F18+$L$3</f>
-        <v>19.296999999999997</v>
-      </c>
-      <c r="E18" s="4"/>
-      <c r="F18" s="3">
-        <v>-16.68</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="13"/>
-      <c r="B19" s="5">
-        <v>922.2</v>
-      </c>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5">
-        <f>F19+$L$4</f>
-        <v>19.333999999999996</v>
-      </c>
-      <c r="E19" s="5"/>
-      <c r="F19" s="3">
-        <v>-16.600000000000001</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="14"/>
-      <c r="B20" s="6">
-        <v>927.8</v>
-      </c>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6">
-        <f>F20+$L$5</f>
-        <v>19.124000000000002</v>
-      </c>
-      <c r="E20" s="6"/>
-      <c r="F20" s="3">
-        <v>-16.68</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10"/>
+      <c r="B10"/>
+      <c r="C10"/>
+      <c r="D10"/>
+      <c r="E10"/>
+      <c r="F10"/>
+    </row>
+    <row r="11" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11"/>
+      <c r="B11"/>
+      <c r="C11"/>
+      <c r="D11"/>
+      <c r="E11"/>
+      <c r="F11"/>
+    </row>
+    <row r="12" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12"/>
+      <c r="B12"/>
+      <c r="C12"/>
+      <c r="D12"/>
+      <c r="E12"/>
+      <c r="F12"/>
+    </row>
+    <row r="13" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13"/>
+      <c r="B13"/>
+      <c r="C13"/>
+      <c r="D13"/>
+      <c r="E13"/>
+      <c r="F13"/>
+    </row>
+    <row r="14" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14"/>
+      <c r="B14"/>
+      <c r="C14"/>
+      <c r="D14"/>
+      <c r="E14"/>
+      <c r="F14"/>
+    </row>
+    <row r="15" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15"/>
+      <c r="B15"/>
+      <c r="C15"/>
+      <c r="D15"/>
+      <c r="E15"/>
+      <c r="F15"/>
+    </row>
+    <row r="16" spans="1:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16"/>
+      <c r="B16"/>
+      <c r="C16"/>
+      <c r="D16"/>
+      <c r="E16"/>
+      <c r="F16"/>
+    </row>
+    <row r="17" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17"/>
+      <c r="B17"/>
+      <c r="C17"/>
+      <c r="D17"/>
+      <c r="E17"/>
+      <c r="F17"/>
+    </row>
+    <row r="18" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18"/>
+      <c r="B18"/>
+      <c r="C18"/>
+      <c r="D18"/>
+      <c r="E18"/>
+      <c r="F18"/>
+    </row>
+    <row r="19" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19"/>
+      <c r="B19"/>
+      <c r="C19"/>
+      <c r="D19"/>
+      <c r="E19"/>
+      <c r="F19"/>
+    </row>
+    <row r="20" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20"/>
+      <c r="B20"/>
+      <c r="C20"/>
+      <c r="D20"/>
+      <c r="E20"/>
+      <c r="F20"/>
+    </row>
+    <row r="21" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21"/>
       <c r="B21"/>
       <c r="C21"/>
       <c r="D21"/>
       <c r="E21"/>
     </row>
-    <row r="22" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22"/>
       <c r="B22"/>
       <c r="C22"/>
       <c r="D22"/>
       <c r="E22"/>
     </row>
-    <row r="23" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23"/>
       <c r="B23"/>
       <c r="C23"/>
       <c r="D23"/>
       <c r="E23"/>
     </row>
-    <row r="24" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24"/>
       <c r="B24"/>
       <c r="C24"/>
@@ -953,23 +832,21 @@
       <c r="E24"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A15:A17"/>
+  <mergeCells count="2">
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="A6:A8"/>
-    <mergeCell ref="A12:A14"/>
-    <mergeCell ref="A18:A20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="7aa56756-527e-4eff-9208-0b4e58a0c97f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1212,20 +1089,17 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="7aa56756-527e-4eff-9208-0b4e58a0c97f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D57F0157-5ABB-467B-BB05-7F492F5F6EF0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D529D985-65F1-4189-89DC-0CE527EC86E5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="7aa56756-527e-4eff-9208-0b4e58a0c97f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1250,9 +1124,11 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D529D985-65F1-4189-89DC-0CE527EC86E5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D57F0157-5ABB-467B-BB05-7F492F5F6EF0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="7aa56756-527e-4eff-9208-0b4e58a0c97f"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>